<commit_message>
DrugSupplyDB V11, ColdChainDB V12
</commit_message>
<xml_diff>
--- a/SourceData/supplychain/LGModData.xlsx
+++ b/SourceData/supplychain/LGModData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proj\SpectrumEngine\DefaultData\SourceData\supplychain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D6845D9-30BA-409D-B0DA-783271506E22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{019C8C00-84EC-4407-AD33-D03CBD577481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{55216F51-A66D-4EBB-A912-BBFA554C2C43}"/>
   </bookViews>
@@ -1777,7 +1777,7 @@
         <v>7452.24</v>
       </c>
       <c r="F2">
-        <v>36</v>
+        <v>3.5999999999999997E-2</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>156</v>
@@ -1800,7 +1800,7 @@
         <v>12360.39</v>
       </c>
       <c r="F3">
-        <v>70</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>156</v>
@@ -1823,7 +1823,7 @@
         <v>5828.51</v>
       </c>
       <c r="F4">
-        <v>57</v>
+        <v>5.7000000000000002E-2</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>156</v>
@@ -1846,7 +1846,7 @@
         <v>6917.73</v>
       </c>
       <c r="F5">
-        <v>102</v>
+        <v>0.10199999999999999</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>156</v>
@@ -1869,7 +1869,7 @@
         <v>4205.3</v>
       </c>
       <c r="F6">
-        <v>37.5</v>
+        <v>3.7499999999999999E-2</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>156</v>
@@ -1892,7 +1892,7 @@
         <v>5800</v>
       </c>
       <c r="F7">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>156</v>
@@ -1915,7 +1915,7 @@
         <v>5830</v>
       </c>
       <c r="F8">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>156</v>
@@ -1938,7 +1938,7 @@
         <v>5870.48</v>
       </c>
       <c r="F9">
-        <v>36</v>
+        <v>3.5999999999999997E-2</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>156</v>
@@ -1961,7 +1961,7 @@
         <v>2550</v>
       </c>
       <c r="F10">
-        <v>48</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>156</v>
@@ -1984,7 +1984,7 @@
         <v>12890.25</v>
       </c>
       <c r="F11">
-        <v>120</v>
+        <v>0.12</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>156</v>
@@ -2007,7 +2007,7 @@
         <v>7155.27</v>
       </c>
       <c r="F12">
-        <v>110</v>
+        <v>0.11</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>156</v>
@@ -2030,7 +2030,7 @@
         <v>5179.6099999999997</v>
       </c>
       <c r="F13">
-        <v>132</v>
+        <v>0.13200000000000001</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>156</v>
@@ -2053,7 +2053,7 @@
         <v>3604.01</v>
       </c>
       <c r="F14">
-        <v>55.5</v>
+        <v>5.5500000000000001E-2</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>156</v>
@@ -2076,7 +2076,7 @@
         <v>4013.9</v>
       </c>
       <c r="F15">
-        <v>92</v>
+        <v>9.1999999999999998E-2</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>156</v>
@@ -2099,7 +2099,7 @@
         <v>5034.76</v>
       </c>
       <c r="F16">
-        <v>170</v>
+        <v>0.17</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>156</v>
@@ -2122,7 +2122,7 @@
         <v>7709.3</v>
       </c>
       <c r="F17">
-        <v>80.5</v>
+        <v>8.0500000000000002E-2</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>156</v>
@@ -2145,7 +2145,7 @@
         <v>2803</v>
       </c>
       <c r="F18">
-        <v>59</v>
+        <v>5.8999999999999997E-2</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>156</v>
@@ -2168,7 +2168,7 @@
         <v>3859.3</v>
       </c>
       <c r="F19">
-        <v>200</v>
+        <v>0.2</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>156</v>
@@ -2191,7 +2191,7 @@
         <v>9260.39</v>
       </c>
       <c r="F20">
-        <v>220</v>
+        <v>0.22</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>156</v>
@@ -2214,7 +2214,7 @@
         <v>3060</v>
       </c>
       <c r="F21">
-        <v>50</v>
+        <v>0.05</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>156</v>
@@ -2237,7 +2237,7 @@
         <v>3455.3</v>
       </c>
       <c r="F22">
-        <v>200</v>
+        <v>0.2</v>
       </c>
       <c r="G22" s="1" t="s">
         <v>156</v>
@@ -3249,7 +3249,7 @@
         <v>1990.73</v>
       </c>
       <c r="F66">
-        <v>52.5</v>
+        <v>5.2499999999999998E-2</v>
       </c>
       <c r="G66" s="1" t="s">
         <v>346</v>
@@ -3272,7 +3272,7 @@
         <v>1500</v>
       </c>
       <c r="F67">
-        <v>50</v>
+        <v>0.05</v>
       </c>
       <c r="G67" s="1" t="s">
         <v>346</v>
@@ -3295,7 +3295,7 @@
         <v>5372.11</v>
       </c>
       <c r="F68">
-        <v>240</v>
+        <v>0.24</v>
       </c>
       <c r="G68" s="1" t="s">
         <v>346</v>
@@ -3318,7 +3318,7 @@
         <v>4259.58</v>
       </c>
       <c r="F69">
-        <v>184</v>
+        <v>0.184</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>346</v>
@@ -3341,7 +3341,7 @@
         <v>968</v>
       </c>
       <c r="F70">
-        <v>61</v>
+        <v>6.0999999999999999E-2</v>
       </c>
       <c r="G70" s="1" t="s">
         <v>346</v>
@@ -3364,7 +3364,7 @@
         <v>1536</v>
       </c>
       <c r="F71">
-        <v>211</v>
+        <v>0.21099999999999999</v>
       </c>
       <c r="G71" s="1" t="s">
         <v>346</v>
@@ -3387,7 +3387,7 @@
         <v>3754.35</v>
       </c>
       <c r="F72">
-        <v>36.5</v>
+        <v>3.6499999999999998E-2</v>
       </c>
       <c r="G72" s="1" t="s">
         <v>346</v>
@@ -3410,7 +3410,7 @@
         <v>4043.86</v>
       </c>
       <c r="F73">
-        <v>80.5</v>
+        <v>8.0500000000000002E-2</v>
       </c>
       <c r="G73" s="1" t="s">
         <v>346</v>
@@ -3433,7 +3433,7 @@
         <v>1733</v>
       </c>
       <c r="F74">
-        <v>30</v>
+        <v>0.03</v>
       </c>
       <c r="G74" s="1" t="s">
         <v>346</v>
@@ -3456,7 +3456,7 @@
         <v>1577.2</v>
       </c>
       <c r="F75">
-        <v>60</v>
+        <v>0.06</v>
       </c>
       <c r="G75" s="1" t="s">
         <v>346</v>
@@ -3479,7 +3479,7 @@
         <v>1722.07</v>
       </c>
       <c r="F76">
-        <v>98</v>
+        <v>9.8000000000000004E-2</v>
       </c>
       <c r="G76" s="1" t="s">
         <v>346</v>
@@ -3502,7 +3502,7 @@
         <v>1986</v>
       </c>
       <c r="F77">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G77" s="1" t="s">
         <v>346</v>
@@ -3525,7 +3525,7 @@
         <v>3221.32</v>
       </c>
       <c r="F78">
-        <v>241</v>
+        <v>0.24099999999999999</v>
       </c>
       <c r="G78" s="1" t="s">
         <v>346</v>
@@ -3548,7 +3548,7 @@
         <v>1507.53</v>
       </c>
       <c r="F79">
-        <v>38</v>
+        <v>3.7999999999999999E-2</v>
       </c>
       <c r="G79" s="1" t="s">
         <v>346</v>
@@ -3571,7 +3571,7 @@
         <v>2685.4</v>
       </c>
       <c r="F80">
-        <v>242</v>
+        <v>0.24199999999999999</v>
       </c>
       <c r="G80" s="1" t="s">
         <v>346</v>
@@ -3594,7 +3594,7 @@
         <v>5704.45</v>
       </c>
       <c r="F81">
-        <v>120</v>
+        <v>0.12</v>
       </c>
       <c r="G81" s="1" t="s">
         <v>346</v>
@@ -3640,7 +3640,7 @@
         <v>86.36</v>
       </c>
       <c r="F83">
-        <v>8</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="G83" s="1" t="s">
         <v>282</v>
@@ -3686,7 +3686,7 @@
         <v>2393</v>
       </c>
       <c r="F85">
-        <v>5.4</v>
+        <v>5.4000000000000003E-3</v>
       </c>
       <c r="G85" s="1" t="s">
         <v>282</v>
@@ -3732,7 +3732,7 @@
         <v>441.48</v>
       </c>
       <c r="F87">
-        <v>6</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="G87" s="1" t="s">
         <v>282</v>
@@ -3755,7 +3755,7 @@
         <v>76.78</v>
       </c>
       <c r="F88">
-        <v>6</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="G88" s="1" t="s">
         <v>282</v>
@@ -3778,7 +3778,7 @@
         <v>106.91</v>
       </c>
       <c r="F89">
-        <v>18</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="G89" s="1" t="s">
         <v>282</v>
@@ -3801,7 +3801,7 @@
         <v>86.36</v>
       </c>
       <c r="F90">
-        <v>5.5</v>
+        <v>5.4999999999999997E-3</v>
       </c>
       <c r="G90" s="1" t="s">
         <v>282</v>
@@ -3824,7 +3824,7 @@
         <v>104.63</v>
       </c>
       <c r="F91">
-        <v>18</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="G91" s="1" t="s">
         <v>282</v>
@@ -3847,7 +3847,7 @@
         <v>104.63</v>
       </c>
       <c r="F92">
-        <v>22.5</v>
+        <v>2.2499999999999999E-2</v>
       </c>
       <c r="G92" s="1" t="s">
         <v>282</v>
@@ -3870,7 +3870,7 @@
         <v>128</v>
       </c>
       <c r="F93">
-        <v>20</v>
+        <v>0.02</v>
       </c>
       <c r="G93" s="1" t="s">
         <v>282</v>
@@ -3893,7 +3893,7 @@
         <v>75</v>
       </c>
       <c r="F94">
-        <v>7</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="G94" s="1" t="s">
         <v>282</v>
@@ -3916,7 +3916,7 @@
         <v>95</v>
       </c>
       <c r="F95">
-        <v>12</v>
+        <v>1.2E-2</v>
       </c>
       <c r="G95" s="1" t="s">
         <v>282</v>
@@ -3939,7 +3939,7 @@
         <v>86.13</v>
       </c>
       <c r="F96">
-        <v>6</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="G96" s="1" t="s">
         <v>282</v>
@@ -3962,7 +3962,7 @@
         <v>73.91</v>
       </c>
       <c r="F97">
-        <v>15</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="G97" s="1" t="s">
         <v>282</v>
@@ -3985,7 +3985,7 @@
         <v>101</v>
       </c>
       <c r="F98">
-        <v>20.25</v>
+        <v>2.0250000000000001E-2</v>
       </c>
       <c r="G98" s="1" t="s">
         <v>282</v>
@@ -4008,7 +4008,7 @@
         <v>84.91</v>
       </c>
       <c r="F99">
-        <v>16</v>
+        <v>1.6E-2</v>
       </c>
       <c r="G99" s="1" t="s">
         <v>282</v>
@@ -4031,7 +4031,7 @@
         <v>719.58</v>
       </c>
       <c r="F100">
-        <v>7</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="G100" s="1" t="s">
         <v>282</v>
@@ -4054,7 +4054,7 @@
         <v>625.72</v>
       </c>
       <c r="F101">
-        <v>20</v>
+        <v>0.02</v>
       </c>
       <c r="G101" s="1" t="s">
         <v>282</v>
@@ -4077,7 +4077,7 @@
         <v>37</v>
       </c>
       <c r="F102">
-        <v>1.6</v>
+        <v>1.6000000000000001E-3</v>
       </c>
       <c r="G102" s="1" t="s">
         <v>282</v>
@@ -4100,7 +4100,7 @@
         <v>239</v>
       </c>
       <c r="F103">
-        <v>15.4</v>
+        <v>1.54E-2</v>
       </c>
       <c r="G103" s="1" t="s">
         <v>282</v>
@@ -4169,7 +4169,7 @@
         <v>47.7</v>
       </c>
       <c r="F106">
-        <v>2.4</v>
+        <v>2.3999999999999998E-3</v>
       </c>
       <c r="G106" s="1" t="s">
         <v>282</v>
@@ -4238,7 +4238,7 @@
         <v>89</v>
       </c>
       <c r="F109">
-        <v>1.8</v>
+        <v>1.8E-3</v>
       </c>
       <c r="G109" s="1" t="s">
         <v>282</v>
@@ -4261,7 +4261,7 @@
         <v>27.96</v>
       </c>
       <c r="F110">
-        <v>1.51</v>
+        <v>1.5100000000000001E-3</v>
       </c>
       <c r="G110" s="1" t="s">
         <v>282</v>
@@ -4307,7 +4307,7 @@
         <v>34</v>
       </c>
       <c r="F112">
-        <v>1.7</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="G112" s="1" t="s">
         <v>282</v>
@@ -4330,7 +4330,7 @@
         <v>28.95</v>
       </c>
       <c r="F113">
-        <v>1.5</v>
+        <v>1.5E-3</v>
       </c>
       <c r="G113" s="1" t="s">
         <v>282</v>
@@ -4376,7 +4376,7 @@
         <v>12.5</v>
       </c>
       <c r="F115">
-        <v>1.7</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="G115" s="1" t="s">
         <v>282</v>
@@ -4399,7 +4399,7 @@
         <v>16</v>
       </c>
       <c r="F116">
-        <v>2.6</v>
+        <v>2.5999999999999999E-3</v>
       </c>
       <c r="G116" s="1" t="s">
         <v>282</v>
@@ -4422,7 +4422,7 @@
         <v>10.75</v>
       </c>
       <c r="F117">
-        <v>1.67</v>
+        <v>1.6699999999999998E-3</v>
       </c>
       <c r="G117" s="1" t="s">
         <v>282</v>
@@ -4445,7 +4445,7 @@
         <v>7.34</v>
       </c>
       <c r="F118">
-        <v>0.9</v>
+        <v>8.9999999999999998E-4</v>
       </c>
       <c r="G118" s="1" t="s">
         <v>282</v>
@@ -4468,7 +4468,7 @@
         <v>12.62</v>
       </c>
       <c r="F119">
-        <v>2.7</v>
+        <v>2.7000000000000001E-3</v>
       </c>
       <c r="G119" s="1" t="s">
         <v>282</v>
@@ -4491,7 +4491,7 @@
         <v>9.15</v>
       </c>
       <c r="F120">
-        <v>1.7</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="G120" s="1" t="s">
         <v>282</v>
@@ -4514,7 +4514,7 @@
         <v>6.69</v>
       </c>
       <c r="F121">
-        <v>0.8</v>
+        <v>8.0000000000000004E-4</v>
       </c>
       <c r="G121" s="1" t="s">
         <v>282</v>
@@ -4537,7 +4537,7 @@
         <v>16.510000000000002</v>
       </c>
       <c r="F122">
-        <v>2.5</v>
+        <v>2.5000000000000001E-3</v>
       </c>
       <c r="G122" s="1" t="s">
         <v>282</v>
@@ -4560,7 +4560,7 @@
         <v>6.86</v>
       </c>
       <c r="F123">
-        <v>0.9</v>
+        <v>8.9999999999999998E-4</v>
       </c>
       <c r="G123" s="1" t="s">
         <v>282</v>
@@ -4583,7 +4583,7 @@
         <v>14.45</v>
       </c>
       <c r="F124">
-        <v>2.9</v>
+        <v>2.8999999999999998E-3</v>
       </c>
       <c r="G124" s="1" t="s">
         <v>282</v>
@@ -4606,7 +4606,7 @@
         <v>17</v>
       </c>
       <c r="F125">
-        <v>3.4</v>
+        <v>3.3999999999999998E-3</v>
       </c>
       <c r="G125" s="1" t="s">
         <v>282</v>

</xml_diff>

<commit_message>
Add LG waste management DB
</commit_message>
<xml_diff>
--- a/SourceData/supplychain/LGModData.xlsx
+++ b/SourceData/supplychain/LGModData.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proj\SpectrumEngine\DefaultData\SourceData\supplychain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{019C8C00-84EC-4407-AD33-D03CBD577481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F14D6B-BDF2-4189-9031-06EC87A709D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{55216F51-A66D-4EBB-A912-BBFA554C2C43}"/>
+    <workbookView xWindow="-23148" yWindow="-1428" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{55216F51-A66D-4EBB-A912-BBFA554C2C43}"/>
   </bookViews>
   <sheets>
     <sheet name="ColdChainDB" sheetId="1" r:id="rId1"/>
+    <sheet name="WasteManagementDB" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="474">
   <si>
     <t>S0005125</t>
   </si>
@@ -1347,13 +1348,127 @@
   </si>
   <si>
     <t>Accessories</t>
+  </si>
+  <si>
+    <t>&lt;Waste Management ID&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Working Life&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Fuel Cost&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Electricity Cost&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Water Cost&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Maint Perc&gt;</t>
+  </si>
+  <si>
+    <t>15-liter bin</t>
+  </si>
+  <si>
+    <t>50-liter bin</t>
+  </si>
+  <si>
+    <t>240-liter wheeled bin</t>
+  </si>
+  <si>
+    <t>24-liter autoclave</t>
+  </si>
+  <si>
+    <t>51-liter autoclave</t>
+  </si>
+  <si>
+    <t>125-liter autoclave</t>
+  </si>
+  <si>
+    <t>340-liter autoclave</t>
+  </si>
+  <si>
+    <t>2300-liter autoclave</t>
+  </si>
+  <si>
+    <t>Simple autoclave shelter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small-scale incinerator (5kg/h) </t>
+  </si>
+  <si>
+    <t>Shelter for small-scale incinerator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small-scale incinerator (12kg/hr) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium-size incinerator (50kg/h) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Large incinerator (350 kg/hr) </t>
+  </si>
+  <si>
+    <t>Shelter for treatment system</t>
+  </si>
+  <si>
+    <t>Sharps pit</t>
+  </si>
+  <si>
+    <t>Small pit</t>
+  </si>
+  <si>
+    <t>Small ash pit</t>
+  </si>
+  <si>
+    <t>Medium ash pit (lined)</t>
+  </si>
+  <si>
+    <t>Large ash pit (lined)</t>
+  </si>
+  <si>
+    <t>Very large ash pit (lined)</t>
+  </si>
+  <si>
+    <t>Medium HCW shredder</t>
+  </si>
+  <si>
+    <t>Large HCW shredder</t>
+  </si>
+  <si>
+    <t>Storage area</t>
+  </si>
+  <si>
+    <t>Large storage area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personal protection equipment </t>
+  </si>
+  <si>
+    <t>Needle remover</t>
+  </si>
+  <si>
+    <t>Reusable sharps containers</t>
+  </si>
+  <si>
+    <t>Transport vehicle (5000 liter capacity)</t>
+  </si>
+  <si>
+    <t>Air pollution control unit</t>
+  </si>
+  <si>
+    <t>&lt;Is Default&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1363,6 +1478,13 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -1387,15 +1509,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -5248,4 +5373,925 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14399450-B815-4255-8C37-457E55D148A4}">
+  <dimension ref="A1:I31"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.5703125" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>437</v>
+      </c>
+      <c r="B1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" t="s">
+        <v>473</v>
+      </c>
+      <c r="D1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" t="s">
+        <v>438</v>
+      </c>
+      <c r="F1" t="s">
+        <v>442</v>
+      </c>
+      <c r="G1" t="s">
+        <v>440</v>
+      </c>
+      <c r="H1" t="s">
+        <v>441</v>
+      </c>
+      <c r="I1" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>443</v>
+      </c>
+      <c r="C2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3">
+        <v>5</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>0.05</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>444</v>
+      </c>
+      <c r="C3" t="b">
+        <v>0</v>
+      </c>
+      <c r="D3" s="3">
+        <v>20</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>0.05</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>445</v>
+      </c>
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3">
+        <v>45</v>
+      </c>
+      <c r="E4">
+        <v>4</v>
+      </c>
+      <c r="F4">
+        <v>0.05</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>446</v>
+      </c>
+      <c r="C5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1000</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5">
+        <v>0.05</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>447</v>
+      </c>
+      <c r="C6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3">
+        <v>1770</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6">
+        <v>0.05</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>448</v>
+      </c>
+      <c r="C7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D7" s="3">
+        <v>31200</v>
+      </c>
+      <c r="E7">
+        <v>10</v>
+      </c>
+      <c r="F7">
+        <v>0.05</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>449</v>
+      </c>
+      <c r="C8" t="b">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3">
+        <v>36500</v>
+      </c>
+      <c r="E8">
+        <v>10</v>
+      </c>
+      <c r="F8">
+        <v>0.05</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>450</v>
+      </c>
+      <c r="C9" t="b">
+        <v>0</v>
+      </c>
+      <c r="D9" s="3">
+        <v>125000</v>
+      </c>
+      <c r="E9">
+        <v>10</v>
+      </c>
+      <c r="F9">
+        <v>0.05</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>451</v>
+      </c>
+      <c r="C10" t="b">
+        <v>0</v>
+      </c>
+      <c r="D10" s="3">
+        <v>300</v>
+      </c>
+      <c r="E10">
+        <v>5</v>
+      </c>
+      <c r="F10">
+        <v>0.05</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>452</v>
+      </c>
+      <c r="C11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11" s="3">
+        <v>1500</v>
+      </c>
+      <c r="E11">
+        <v>3</v>
+      </c>
+      <c r="F11">
+        <v>0.05</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>453</v>
+      </c>
+      <c r="C12" t="b">
+        <v>0</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1000</v>
+      </c>
+      <c r="E12">
+        <v>5</v>
+      </c>
+      <c r="F12">
+        <v>0.05</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>454</v>
+      </c>
+      <c r="C13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3">
+        <v>2800</v>
+      </c>
+      <c r="E13">
+        <v>5</v>
+      </c>
+      <c r="F13">
+        <v>0.05</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>455</v>
+      </c>
+      <c r="C14" t="b">
+        <v>0</v>
+      </c>
+      <c r="D14" s="3">
+        <v>37500</v>
+      </c>
+      <c r="E14">
+        <v>10</v>
+      </c>
+      <c r="F14">
+        <v>0.05</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>456</v>
+      </c>
+      <c r="C15" t="b">
+        <v>0</v>
+      </c>
+      <c r="D15" s="3">
+        <v>200000</v>
+      </c>
+      <c r="E15">
+        <v>10</v>
+      </c>
+      <c r="F15">
+        <v>0.05</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>457</v>
+      </c>
+      <c r="C16" t="b">
+        <v>0</v>
+      </c>
+      <c r="D16" s="3">
+        <v>2000</v>
+      </c>
+      <c r="E16">
+        <v>10</v>
+      </c>
+      <c r="F16">
+        <v>0.05</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>458</v>
+      </c>
+      <c r="C17" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" s="3">
+        <v>100</v>
+      </c>
+      <c r="E17">
+        <v>5</v>
+      </c>
+      <c r="F17">
+        <v>0.05</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>459</v>
+      </c>
+      <c r="C18" t="b">
+        <v>0</v>
+      </c>
+      <c r="D18" s="3">
+        <v>25</v>
+      </c>
+      <c r="E18">
+        <v>2</v>
+      </c>
+      <c r="F18">
+        <v>0.05</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>460</v>
+      </c>
+      <c r="C19" t="b">
+        <v>1</v>
+      </c>
+      <c r="D19" s="3">
+        <v>25</v>
+      </c>
+      <c r="E19">
+        <v>5</v>
+      </c>
+      <c r="F19">
+        <v>0.05</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>461</v>
+      </c>
+      <c r="C20" t="b">
+        <v>0</v>
+      </c>
+      <c r="D20" s="3">
+        <v>250</v>
+      </c>
+      <c r="E20">
+        <v>5</v>
+      </c>
+      <c r="F20">
+        <v>0.05</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>462</v>
+      </c>
+      <c r="C21" t="b">
+        <v>0</v>
+      </c>
+      <c r="D21" s="3">
+        <v>250</v>
+      </c>
+      <c r="E21">
+        <v>3</v>
+      </c>
+      <c r="F21">
+        <v>0.05</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>463</v>
+      </c>
+      <c r="C22" t="b">
+        <v>0</v>
+      </c>
+      <c r="D22" s="3">
+        <v>500</v>
+      </c>
+      <c r="E22">
+        <v>2</v>
+      </c>
+      <c r="F22">
+        <v>0.05</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>464</v>
+      </c>
+      <c r="C23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D23" s="3">
+        <v>25000</v>
+      </c>
+      <c r="E23">
+        <v>5</v>
+      </c>
+      <c r="F23">
+        <v>0.05</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>465</v>
+      </c>
+      <c r="C24" t="b">
+        <v>0</v>
+      </c>
+      <c r="D24" s="3">
+        <v>56000</v>
+      </c>
+      <c r="E24">
+        <v>5</v>
+      </c>
+      <c r="F24">
+        <v>0.05</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>466</v>
+      </c>
+      <c r="C25" t="b">
+        <v>1</v>
+      </c>
+      <c r="D25" s="3">
+        <v>1000</v>
+      </c>
+      <c r="E25">
+        <v>10</v>
+      </c>
+      <c r="F25">
+        <v>0.05</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>467</v>
+      </c>
+      <c r="C26" t="b">
+        <v>0</v>
+      </c>
+      <c r="D26" s="3">
+        <v>2000</v>
+      </c>
+      <c r="E26">
+        <v>10</v>
+      </c>
+      <c r="F26">
+        <v>0.05</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>468</v>
+      </c>
+      <c r="C27" t="b">
+        <v>1</v>
+      </c>
+      <c r="D27" s="3">
+        <v>35</v>
+      </c>
+      <c r="E27">
+        <v>2</v>
+      </c>
+      <c r="F27">
+        <v>0.05</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>469</v>
+      </c>
+      <c r="C28" t="b">
+        <v>0</v>
+      </c>
+      <c r="D28" s="3">
+        <v>30</v>
+      </c>
+      <c r="E28">
+        <v>4</v>
+      </c>
+      <c r="F28">
+        <v>0.05</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>0</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>470</v>
+      </c>
+      <c r="C29" t="b">
+        <v>1</v>
+      </c>
+      <c r="D29" s="3">
+        <v>35</v>
+      </c>
+      <c r="E29">
+        <v>2</v>
+      </c>
+      <c r="F29">
+        <v>0.05</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29">
+        <v>0</v>
+      </c>
+      <c r="I29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>471</v>
+      </c>
+      <c r="C30" t="b">
+        <v>0</v>
+      </c>
+      <c r="D30" s="3">
+        <v>40000</v>
+      </c>
+      <c r="E30">
+        <v>5</v>
+      </c>
+      <c r="F30">
+        <v>0.05</v>
+      </c>
+      <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="H30">
+        <v>0</v>
+      </c>
+      <c r="I30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>472</v>
+      </c>
+      <c r="C31" t="b">
+        <v>0</v>
+      </c>
+      <c r="D31" s="3">
+        <v>286000</v>
+      </c>
+      <c r="E31">
+        <v>10</v>
+      </c>
+      <c r="F31">
+        <v>0.05</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31">
+        <v>0</v>
+      </c>
+      <c r="I31">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>